<commit_message>
Fix: swap 2023/2024 columns in Balance Sheet
</commit_message>
<xml_diff>
--- a/FinAnalyst.xlsx
+++ b/FinAnalyst.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/16b66fb0cd5197bd/Desktop/FinancialAnalyzer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="490" documentId="8_{940DF5F5-D8F3-4AD4-B054-56665D0CBCC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9551758A-53D0-4DF9-A558-166C8AB2A854}"/>
+  <xr:revisionPtr revIDLastSave="495" documentId="8_{940DF5F5-D8F3-4AD4-B054-56665D0CBCC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64090363-FCA9-4D50-9C65-C27EFADA8FAB}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{84B09E3A-B350-4F10-AB78-3897FE5FB26D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{84B09E3A-B350-4F10-AB78-3897FE5FB26D}"/>
   </bookViews>
   <sheets>
     <sheet name="Income Statement" sheetId="1" r:id="rId1"/>
@@ -3321,8 +3321,8 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="76.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="8.88671875" style="2"/>
-    <col min="6" max="6" width="8.88671875" style="2"/>
+    <col min="2" max="2" width="8.88671875" style="2"/>
+    <col min="5" max="5" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.3">
@@ -3358,10 +3358,10 @@
         <v>2025</v>
       </c>
       <c r="C2" s="6">
+        <v>2024</v>
+      </c>
+      <c r="D2" s="6">
         <v>2023</v>
-      </c>
-      <c r="D2" s="6">
-        <v>2024</v>
       </c>
       <c r="E2" s="6">
         <v>2022</v>
@@ -3458,10 +3458,10 @@
         <v>467</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>544</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>468</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>117</v>
@@ -3558,10 +3558,10 @@
         <v>469</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>545</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>470</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>119</v>
@@ -3602,10 +3602,10 @@
         <v>471</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>546</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>472</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>121</v>
@@ -3646,10 +3646,10 @@
         <v>473</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>547</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>474</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>123</v>
@@ -3690,10 +3690,10 @@
         <v>363</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>548</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>475</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>125</v>
@@ -3760,10 +3760,10 @@
         <v>476</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>549</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>477</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>127</v>
@@ -3832,10 +3832,10 @@
         <v>478</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>550</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>479</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>129</v>
@@ -3876,10 +3876,10 @@
         <v>480</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>551</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>295</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>131</v>
@@ -3920,10 +3920,10 @@
         <v>481</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>552</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>482</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>133</v>
@@ -3964,10 +3964,10 @@
         <v>483</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>553</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>484</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>135</v>
@@ -4036,10 +4036,10 @@
         <v>485</v>
       </c>
       <c r="C20" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>554</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>486</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>137</v>
@@ -4080,10 +4080,10 @@
         <v>487</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>555</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>488</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>139</v>
@@ -4124,10 +4124,10 @@
         <v>489</v>
       </c>
       <c r="C22" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>556</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>490</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>141</v>
@@ -4196,10 +4196,10 @@
         <v>491</v>
       </c>
       <c r="C24" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>557</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>492</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>143</v>
@@ -4240,10 +4240,10 @@
         <v>493</v>
       </c>
       <c r="C25" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>333</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>494</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>145</v>
@@ -4284,10 +4284,10 @@
         <v>495</v>
       </c>
       <c r="C26" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>558</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>496</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>147</v>
@@ -4328,10 +4328,10 @@
         <v>497</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>493</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>498</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>149</v>
@@ -4372,10 +4372,10 @@
         <v>499</v>
       </c>
       <c r="C28" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>559</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>500</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>151</v>
@@ -4416,10 +4416,10 @@
         <v>501</v>
       </c>
       <c r="C29" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>560</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>502</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>153</v>
@@ -4460,10 +4460,10 @@
         <v>503</v>
       </c>
       <c r="C30" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>561</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>504</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>155</v>
@@ -4560,10 +4560,10 @@
         <v>505</v>
       </c>
       <c r="C33" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="D33" s="1" t="s">
         <v>562</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>506</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>157</v>
@@ -4604,10 +4604,10 @@
         <v>507</v>
       </c>
       <c r="C34" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>563</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>508</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>157</v>
@@ -4676,10 +4676,10 @@
         <v>509</v>
       </c>
       <c r="C36" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="D36" s="1" t="s">
         <v>564</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>510</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>160</v>
@@ -4720,10 +4720,10 @@
         <v>511</v>
       </c>
       <c r="C37" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="D37" s="1" t="s">
         <v>565</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>512</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>162</v>
@@ -4764,10 +4764,10 @@
         <v>513</v>
       </c>
       <c r="C38" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>566</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>260</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>164</v>
@@ -4808,10 +4808,10 @@
         <v>514</v>
       </c>
       <c r="C39" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>389</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>515</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>166</v>
@@ -4878,10 +4878,10 @@
         <v>516</v>
       </c>
       <c r="C41" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="D41" s="1" t="s">
         <v>567</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>517</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>168</v>
@@ -4950,10 +4950,10 @@
         <v>518</v>
       </c>
       <c r="C43" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="D43" s="1" t="s">
         <v>568</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>519</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>170</v>
@@ -4994,10 +4994,10 @@
         <v>520</v>
       </c>
       <c r="C44" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="D44" s="1" t="s">
         <v>569</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>521</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>172</v>
@@ -5066,10 +5066,10 @@
         <v>522</v>
       </c>
       <c r="C46" s="1" t="s">
+        <v>523</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>460</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>523</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>174</v>
@@ -5110,10 +5110,10 @@
         <v>524</v>
       </c>
       <c r="C47" s="1" t="s">
+        <v>525</v>
+      </c>
+      <c r="D47" s="1" t="s">
         <v>570</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>525</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>176</v>
@@ -5154,10 +5154,10 @@
         <v>526</v>
       </c>
       <c r="C48" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="D48" s="1" t="s">
         <v>571</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>527</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>178</v>
@@ -5198,10 +5198,10 @@
         <v>528</v>
       </c>
       <c r="C49" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="D49" s="1" t="s">
         <v>572</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>529</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>180</v>
@@ -5242,10 +5242,10 @@
         <v>530</v>
       </c>
       <c r="C50" s="1" t="s">
+        <v>531</v>
+      </c>
+      <c r="D50" s="1" t="s">
         <v>573</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>531</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>182</v>
@@ -5286,10 +5286,10 @@
         <v>532</v>
       </c>
       <c r="C51" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="D51" s="1" t="s">
         <v>574</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>533</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>184</v>
@@ -5430,10 +5430,10 @@
         <v>534</v>
       </c>
       <c r="C55" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="D55" s="1" t="s">
         <v>575</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>535</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>187</v>
@@ -5474,10 +5474,10 @@
         <v>536</v>
       </c>
       <c r="C56" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="D56" s="1" t="s">
         <v>576</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>537</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>189</v>
@@ -5518,10 +5518,10 @@
         <v>-7660</v>
       </c>
       <c r="C57" s="1">
+        <v>-8110</v>
+      </c>
+      <c r="D57" s="1">
         <v>-7681</v>
-      </c>
-      <c r="D57" s="1">
-        <v>-8110</v>
       </c>
       <c r="E57" s="1">
         <v>-7139</v>
@@ -5600,10 +5600,10 @@
         <v>-4233</v>
       </c>
       <c r="C59" s="1">
+        <v>-4655</v>
+      </c>
+      <c r="D59" s="1">
         <v>-4374</v>
-      </c>
-      <c r="D59" s="1">
-        <v>-4655</v>
       </c>
       <c r="E59" s="1">
         <v>-3871</v>
@@ -5644,10 +5644,10 @@
         <v>538</v>
       </c>
       <c r="C60" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="D60" s="1" t="s">
         <v>577</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>539</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>192</v>
@@ -5688,10 +5688,10 @@
         <v>540</v>
       </c>
       <c r="C61" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="D61" s="1" t="s">
         <v>578</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>541</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>194</v>
@@ -5732,10 +5732,10 @@
         <v>542</v>
       </c>
       <c r="C62" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>579</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>543</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>196</v>
@@ -5776,10 +5776,10 @@
         <v>503</v>
       </c>
       <c r="C63" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="D63" s="1" t="s">
         <v>561</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>504</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>155</v>
@@ -5813,6 +5813,7 @@
       <c r="Y63" s="1"/>
     </row>
     <row r="64" spans="1:25" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L64" s="1"/>
       <c r="M64" s="1"/>
       <c r="N64" s="1"/>
       <c r="O64" s="1"/>
@@ -5825,9 +5826,9 @@
       <c r="V64" s="1"/>
       <c r="W64" s="1"/>
       <c r="X64" s="1"/>
-      <c r="Y64" s="1"/>
-    </row>
-    <row r="65" spans="13:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="65" spans="12:24" x14ac:dyDescent="0.3">
+      <c r="L65" s="1"/>
       <c r="M65" s="1"/>
       <c r="N65" s="1"/>
       <c r="O65" s="1"/>
@@ -5840,9 +5841,9 @@
       <c r="V65" s="1"/>
       <c r="W65" s="1"/>
       <c r="X65" s="1"/>
-      <c r="Y65" s="1"/>
-    </row>
-    <row r="66" spans="13:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="66" spans="12:24" x14ac:dyDescent="0.3">
+      <c r="L66" s="1"/>
       <c r="M66" s="1"/>
       <c r="N66" s="1"/>
       <c r="O66" s="1"/>
@@ -5855,9 +5856,9 @@
       <c r="V66" s="1"/>
       <c r="W66" s="1"/>
       <c r="X66" s="1"/>
-      <c r="Y66" s="1"/>
-    </row>
-    <row r="67" spans="13:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="67" spans="12:24" x14ac:dyDescent="0.3">
+      <c r="L67" s="1"/>
       <c r="M67" s="1"/>
       <c r="N67" s="1"/>
       <c r="O67" s="1"/>
@@ -5870,9 +5871,9 @@
       <c r="V67" s="1"/>
       <c r="W67" s="1"/>
       <c r="X67" s="1"/>
-      <c r="Y67" s="1"/>
-    </row>
-    <row r="68" spans="13:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="68" spans="12:24" x14ac:dyDescent="0.3">
+      <c r="L68" s="1"/>
       <c r="M68" s="1"/>
       <c r="N68" s="1"/>
       <c r="O68" s="1"/>
@@ -5885,9 +5886,9 @@
       <c r="V68" s="1"/>
       <c r="W68" s="1"/>
       <c r="X68" s="1"/>
-      <c r="Y68" s="1"/>
-    </row>
-    <row r="69" spans="13:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="69" spans="12:24" x14ac:dyDescent="0.3">
+      <c r="L69" s="1"/>
       <c r="M69" s="1"/>
       <c r="N69" s="1"/>
       <c r="O69" s="1"/>
@@ -5900,9 +5901,9 @@
       <c r="V69" s="1"/>
       <c r="W69" s="1"/>
       <c r="X69" s="1"/>
-      <c r="Y69" s="1"/>
-    </row>
-    <row r="70" spans="13:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="70" spans="12:24" x14ac:dyDescent="0.3">
+      <c r="L70" s="1"/>
       <c r="M70" s="1"/>
       <c r="N70" s="1"/>
       <c r="O70" s="1"/>
@@ -5915,9 +5916,9 @@
       <c r="V70" s="1"/>
       <c r="W70" s="1"/>
       <c r="X70" s="1"/>
-      <c r="Y70" s="1"/>
-    </row>
-    <row r="71" spans="13:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="71" spans="12:24" x14ac:dyDescent="0.3">
+      <c r="L71" s="1"/>
       <c r="M71" s="1"/>
       <c r="N71" s="1"/>
       <c r="O71" s="1"/>
@@ -5930,9 +5931,9 @@
       <c r="V71" s="1"/>
       <c r="W71" s="1"/>
       <c r="X71" s="1"/>
-      <c r="Y71" s="1"/>
-    </row>
-    <row r="72" spans="13:25" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="72" spans="12:24" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L72" s="1"/>
       <c r="M72" s="1"/>
       <c r="N72" s="1"/>
       <c r="O72" s="1"/>
@@ -5945,9 +5946,9 @@
       <c r="V72" s="1"/>
       <c r="W72" s="1"/>
       <c r="X72" s="1"/>
-      <c r="Y72" s="1"/>
-    </row>
-    <row r="73" spans="13:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="73" spans="12:24" x14ac:dyDescent="0.3">
+      <c r="L73" s="1"/>
       <c r="M73" s="1"/>
       <c r="N73" s="1"/>
       <c r="O73" s="1"/>
@@ -5960,9 +5961,9 @@
       <c r="V73" s="1"/>
       <c r="W73" s="1"/>
       <c r="X73" s="1"/>
-      <c r="Y73" s="1"/>
-    </row>
-    <row r="74" spans="13:25" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="74" spans="12:24" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L74" s="1"/>
       <c r="M74" s="1"/>
       <c r="N74" s="1"/>
       <c r="O74" s="1"/>
@@ -5975,9 +5976,9 @@
       <c r="V74" s="1"/>
       <c r="W74" s="1"/>
       <c r="X74" s="1"/>
-      <c r="Y74" s="1"/>
-    </row>
-    <row r="75" spans="13:25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="75" spans="12:24" x14ac:dyDescent="0.3">
+      <c r="L75" s="1"/>
       <c r="M75" s="1"/>
       <c r="N75" s="1"/>
       <c r="O75" s="1"/>
@@ -5990,10 +5991,9 @@
       <c r="V75" s="1"/>
       <c r="W75" s="1"/>
       <c r="X75" s="1"/>
-      <c r="Y75" s="1"/>
-    </row>
-    <row r="76" spans="13:25" ht="16.2" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="78" spans="13:25" ht="25.8" customHeight="1" x14ac:dyDescent="0.3"/>
+    </row>
+    <row r="76" spans="12:24" ht="16.2" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="78" spans="12:24" ht="25.8" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="82" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="84" ht="16.2" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="86" ht="16.2" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>